<commit_message>
EndLoop - LipSync 기능 추가
DefaultLip 하드코딩에서 데이터 문서화하여 아이돌별로 관리하도록 변경
LipSync 시에 아이돌 및 트랙 키워드 기반으로 데이터 참조하여 동작하도록 수정
</commit_message>
<xml_diff>
--- a/resource/Script/ScriptManual.xlsx
+++ b/resource/Script/ScriptManual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\usosctheater\resource\Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480F613F-6152-4B8A-A5D4-6447C0B0071E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2762FDBF-85A5-4108-B10E-2982731A1CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{F190326C-52FC-4B9A-869B-607708A8B8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{F190326C-52FC-4B9A-869B-607708A8B8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="ScriptManual" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="559">
   <si>
     <t>* 본 문서는 가짜샤니마스극장의 스크립트에 사용할 스크립트 전용 제작 시트입니다.</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -2073,6 +2073,14 @@
   </si>
   <si>
     <t>BGM_77</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>* 메이 무표정으로 말할 때에는 lip_surp 쓰세요</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>* 사히 무표정으로 말할 때에는 lip_surp 쓰세요</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -2080,7 +2088,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <color theme="1"/>
@@ -2179,6 +2187,13 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="넥슨Lv2고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -2243,7 +2258,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2296,6 +2311,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -7002,11 +7020,8 @@
       <c r="E22" t="s">
         <v>69</v>
       </c>
-      <c r="G22" t="s">
-        <v>65</v>
-      </c>
-      <c r="J22" t="s">
-        <v>72</v>
+      <c r="G22" s="18" t="s">
+        <v>557</v>
       </c>
       <c r="M22" t="s">
         <v>183</v>
@@ -7022,12 +7037,6 @@
       <c r="E23" t="s">
         <v>70</v>
       </c>
-      <c r="G23" t="s">
-        <v>66</v>
-      </c>
-      <c r="J23" t="s">
-        <v>73</v>
-      </c>
       <c r="M23" t="s">
         <v>281</v>
       </c>
@@ -7042,12 +7051,6 @@
       <c r="E24" t="s">
         <v>84</v>
       </c>
-      <c r="G24" t="s">
-        <v>86</v>
-      </c>
-      <c r="J24" t="s">
-        <v>87</v>
-      </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
@@ -7057,16 +7060,13 @@
         <v>144</v>
       </c>
       <c r="G25" t="s">
-        <v>139</v>
+        <v>65</v>
       </c>
       <c r="J25" t="s">
-        <v>140</v>
-      </c>
-      <c r="M25" t="s">
-        <v>90</v>
-      </c>
-      <c r="P25" t="s">
-        <v>91</v>
+        <v>72</v>
+      </c>
+      <c r="M25" s="18" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.3">
@@ -7077,16 +7077,16 @@
         <v>149</v>
       </c>
       <c r="G26" t="s">
-        <v>145</v>
+        <v>66</v>
       </c>
       <c r="J26" t="s">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="M26" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="P26" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
@@ -7096,11 +7096,17 @@
       <c r="E27" t="s">
         <v>151</v>
       </c>
+      <c r="G27" t="s">
+        <v>86</v>
+      </c>
+      <c r="J27" t="s">
+        <v>87</v>
+      </c>
       <c r="M27" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="P27" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
@@ -7110,11 +7116,17 @@
       <c r="E28" t="s">
         <v>179</v>
       </c>
+      <c r="G28" t="s">
+        <v>139</v>
+      </c>
+      <c r="J28" t="s">
+        <v>140</v>
+      </c>
       <c r="M28" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="P28" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
@@ -7124,11 +7136,17 @@
       <c r="E29" t="s">
         <v>181</v>
       </c>
+      <c r="G29" t="s">
+        <v>145</v>
+      </c>
+      <c r="J29" t="s">
+        <v>146</v>
+      </c>
       <c r="M29" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="P29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
@@ -7139,10 +7157,10 @@
         <v>185</v>
       </c>
       <c r="M30" t="s">
-        <v>141</v>
+        <v>82</v>
       </c>
       <c r="P30" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.3">
@@ -7153,10 +7171,10 @@
         <v>186</v>
       </c>
       <c r="M31" t="s">
-        <v>300</v>
+        <v>141</v>
       </c>
       <c r="P31" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.3">
@@ -7165,6 +7183,12 @@
       </c>
       <c r="E32" t="s">
         <v>187</v>
+      </c>
+      <c r="M32" t="s">
+        <v>300</v>
+      </c>
+      <c r="P32" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>